<commit_message>
depot menu change commit
</commit_message>
<xml_diff>
--- a/VMS_SOURCE/Templates/RawMeterialProcurementReportTemplate.xlsx
+++ b/VMS_SOURCE/Templates/RawMeterialProcurementReportTemplate.xlsx
@@ -12,14 +12,15 @@
     <workbookView xWindow="96" yWindow="156" windowWidth="20736" windowHeight="9240"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Summary" sheetId="1" r:id="rId1"/>
+    <sheet name="Details" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="124519" calcOnSave="0" concurrentCalc="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="18">
   <si>
     <t>Raw Material Procurement Report Report</t>
   </si>
@@ -30,12 +31,6 @@
     <t>Vendor Name</t>
   </si>
   <si>
-    <t>RM Code</t>
-  </si>
-  <si>
-    <t>RM Name</t>
-  </si>
-  <si>
     <t>Request Id</t>
   </si>
   <si>
@@ -64,6 +59,21 @@
   </si>
   <si>
     <t>Received Date</t>
+  </si>
+  <si>
+    <t>RM Vendor Code</t>
+  </si>
+  <si>
+    <t>RM Vendor Name</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Request Raw Material </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Despatch Raw Material </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Received Raw Material </t>
   </si>
 </sst>
 </file>
@@ -501,40 +511,40 @@
         <v>2</v>
       </c>
       <c r="C2" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="E2" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="D2" s="1" t="s">
+      <c r="F2" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="E2" s="1" t="s">
+      <c r="G2" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="F2" s="1" t="s">
+      <c r="H2" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="G2" s="1" t="s">
+      <c r="I2" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="H2" s="1" t="s">
+      <c r="J2" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="I2" s="1" t="s">
+      <c r="K2" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="J2" s="1" t="s">
+      <c r="L2" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="M2" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="K2" s="2" t="s">
+      <c r="N2" s="2" t="s">
         <v>11</v>
-      </c>
-      <c r="L2" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="M2" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="N2" s="2" t="s">
-        <v>13</v>
       </c>
     </row>
   </sheetData>
@@ -544,4 +554,109 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:Q2"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="12" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="27.44140625" customWidth="1"/>
+    <col min="3" max="3" width="15.44140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="26.109375" customWidth="1"/>
+    <col min="5" max="5" width="9" customWidth="1"/>
+    <col min="6" max="6" width="12.21875" customWidth="1"/>
+    <col min="7" max="7" width="11.109375" customWidth="1"/>
+    <col min="8" max="8" width="51" customWidth="1"/>
+    <col min="9" max="9" width="8.77734375" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="12.6640625" customWidth="1"/>
+    <col min="11" max="11" width="8.77734375" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="39.44140625" customWidth="1"/>
+    <col min="14" max="14" width="12.33203125" customWidth="1"/>
+    <col min="15" max="15" width="11.5546875" customWidth="1"/>
+    <col min="16" max="16" width="29.44140625" customWidth="1"/>
+    <col min="17" max="17" width="11.5546875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:17" ht="18" x14ac:dyDescent="0.3">
+      <c r="A1" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="3"/>
+      <c r="C1" s="3"/>
+      <c r="D1" s="3"/>
+      <c r="E1" s="3"/>
+      <c r="F1" s="3"/>
+      <c r="G1" s="3"/>
+      <c r="H1" s="3"/>
+      <c r="I1" s="3"/>
+      <c r="J1" s="3"/>
+      <c r="K1" s="3"/>
+      <c r="L1" s="3"/>
+      <c r="M1" s="3"/>
+      <c r="N1" s="3"/>
+      <c r="O1" s="3"/>
+      <c r="P1" s="3"/>
+      <c r="Q1" s="3"/>
+    </row>
+    <row r="2" spans="1:17" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A2" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="G2" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="H2" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="I2" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="J2" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="K2" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="L2" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="M2" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="N2" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="O2" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="P2" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="Q2" s="2" t="s">
+        <v>11</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:Q1"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>